<commit_message>
Vidage du fichier import_prospects.xlsx dans public/docs
</commit_message>
<xml_diff>
--- a/public/docs/import_prospects.xlsx
+++ b/public/docs/import_prospects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\FADWA\ERP\api_0.1\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95341B9-CEC3-4781-890F-F2BE9A2F4B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F0A2C9-AEDA-444C-AF76-C77AEEE79486}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="50" yWindow="1900" windowWidth="19150" windowHeight="7360" xr2:uid="{9D75755E-FE6E-4BAB-BDD4-4CD9ECED924A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{9D75755E-FE6E-4BAB-BDD4-4CD9ECED924A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>cin</t>
   </si>
@@ -48,31 +48,7 @@
     <t>ville</t>
   </si>
   <si>
-    <t>cin_25</t>
-  </si>
-  <si>
-    <t>n-1</t>
-  </si>
-  <si>
-    <t>p-1</t>
-  </si>
-  <si>
-    <t>n-1@gmail.com</t>
-  </si>
-  <si>
-    <t>meknes</t>
-  </si>
-  <si>
     <t>source</t>
-  </si>
-  <si>
-    <t>Avito</t>
-  </si>
-  <si>
-    <t>+212678985544</t>
-  </si>
-  <si>
-    <t>+212678655997</t>
   </si>
   <si>
     <t>partenaire</t>
@@ -476,43 +452,19 @@
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>7</v>
-      </c>
-      <c r="B2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H2" t="s">
-        <v>13</v>
-      </c>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="3"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" xr:uid="{95488E9E-1B8F-433E-9BC8-301612A07745}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>